<commit_message>
authoring full draft workflow
</commit_message>
<xml_diff>
--- a/registry/DEEP_Agent_문서분류_레지스트리_v2.2.xlsx
+++ b/registry/DEEP_Agent_문서분류_레지스트리_v2.2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lsh930309/projects/dataFatory/registry/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68BD08CF-45D2-0D49-8161-DD7796FDF0C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C6EA8D6-3D14-9E4B-9326-E3CAC7F40F85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21800" yWindow="-28200" windowWidth="51200" windowHeight="28200" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16920" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0.안내" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3183" uniqueCount="828">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3184" uniqueCount="829">
   <si>
     <t>DEEP Agent 문서 분류 레지스트리 — 데이터 대시보드</t>
   </si>
@@ -2529,6 +2529,10 @@
   </si>
   <si>
     <t>잔액증명서</t>
+  </si>
+  <si>
+    <t>교체필요</t>
+    <phoneticPr fontId="27" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -2538,7 +2542,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2724,6 +2728,13 @@
       <family val="3"/>
       <charset val="129"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Malgun Gothic"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -2847,7 +2858,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3036,18 +3047,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -3334,7 +3348,7 @@
       <c r="F2" s="65"/>
     </row>
     <row r="3" spans="2:6">
-      <c r="B3" s="66" t="s">
+      <c r="B3" s="67" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="65"/>
@@ -3343,7 +3357,7 @@
       <c r="F3" s="65"/>
     </row>
     <row r="4" spans="2:6">
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="66" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="65"/>
@@ -3352,7 +3366,7 @@
       <c r="F4" s="65"/>
     </row>
     <row r="6" spans="2:6" ht="20" customHeight="1">
-      <c r="B6" s="67" t="s">
+      <c r="B6" s="64" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="65"/>
@@ -3436,7 +3450,7 @@
       </c>
     </row>
     <row r="13" spans="2:6" ht="20" customHeight="1">
-      <c r="B13" s="67" t="s">
+      <c r="B13" s="64" t="s">
         <v>14</v>
       </c>
       <c r="C13" s="65"/>
@@ -3476,7 +3490,7 @@
       </c>
     </row>
     <row r="18" spans="2:4" ht="20" customHeight="1">
-      <c r="B18" s="67" t="s">
+      <c r="B18" s="64" t="s">
         <v>20</v>
       </c>
       <c r="C18" s="65"/>
@@ -3549,7 +3563,7 @@
       </c>
     </row>
     <row r="26" spans="2:4" ht="20" customHeight="1">
-      <c r="B26" s="67" t="s">
+      <c r="B26" s="64" t="s">
         <v>26</v>
       </c>
       <c r="C26" s="65"/>
@@ -3644,7 +3658,7 @@
       </c>
     </row>
     <row r="36" spans="2:4" ht="20" customHeight="1">
-      <c r="B36" s="67" t="s">
+      <c r="B36" s="64" t="s">
         <v>34</v>
       </c>
       <c r="C36" s="65"/>
@@ -3750,7 +3764,7 @@
       </c>
     </row>
     <row r="47" spans="2:4" ht="20" customHeight="1">
-      <c r="B47" s="67" t="s">
+      <c r="B47" s="64" t="s">
         <v>43</v>
       </c>
       <c r="C47" s="65"/>
@@ -3823,7 +3837,7 @@
       </c>
     </row>
     <row r="55" spans="2:4" ht="20" customHeight="1">
-      <c r="B55" s="67" t="s">
+      <c r="B55" s="64" t="s">
         <v>49</v>
       </c>
       <c r="C55" s="65"/>
@@ -3885,7 +3899,7 @@
       </c>
     </row>
     <row r="62" spans="2:4" ht="20" customHeight="1">
-      <c r="B62" s="67" t="s">
+      <c r="B62" s="64" t="s">
         <v>53</v>
       </c>
       <c r="C62" s="65"/>
@@ -4035,7 +4049,7 @@
       </c>
     </row>
     <row r="77" spans="2:4" ht="20" customHeight="1">
-      <c r="B77" s="67" t="s">
+      <c r="B77" s="64" t="s">
         <v>66</v>
       </c>
       <c r="C77" s="65"/>
@@ -4218,7 +4232,7 @@
       </c>
     </row>
     <row r="95" spans="2:6" ht="20" customHeight="1">
-      <c r="B95" s="67" t="s">
+      <c r="B95" s="64" t="s">
         <v>82</v>
       </c>
       <c r="C95" s="65"/>
@@ -4305,11 +4319,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B95:F95"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B77:D77"/>
-    <mergeCell ref="B4:F4"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="C102:F102"/>
@@ -4325,6 +4334,11 @@
     <mergeCell ref="B62:D62"/>
     <mergeCell ref="C99:F99"/>
     <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B95:F95"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B77:D77"/>
+    <mergeCell ref="B4:F4"/>
   </mergeCells>
   <phoneticPr fontId="27" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14497,7 +14511,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="16">
+    <row r="25" spans="1:6" ht="18">
       <c r="A25" s="52" t="s">
         <v>220</v>
       </c>
@@ -14513,7 +14527,9 @@
       <c r="E25" s="52" t="s">
         <v>778</v>
       </c>
-      <c r="F25" s="52"/>
+      <c r="F25" s="72" t="s">
+        <v>828</v>
+      </c>
     </row>
     <row r="26" spans="1:6" ht="16">
       <c r="A26" s="52" t="s">

</xml_diff>